<commit_message>
fix: restore sub-district data lost in v2 and correct Bueng Kan codes
Restore the tambon additions, removals and corrections from PR #20 that
were dropped when data/raw was rebuilt for v2, checked against the DOPA
location codes (04/01/2566):

- add 22 sub-districts (21 Bangkok khwaeng, ท่าแฝก under น้ำปาด)
- remove 38 rows for tambons that moved to newer districts or no longer exist
- correct 5 Thai names and 14 English names
- update 41 zip codes confirmed against Thailand Post's post office list;
  27 PR #20 zip changes that could not be confirmed are left unchanged
- put Bueng Kan district names on their DOPA codes and renumber its
  sub-districts to DOPA codes (restores ตำบลสมสนุก)

Refs #45
Closes #43

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/formats/xlsx/districts.xlsx
+++ b/formats/xlsx/districts.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,37 +417,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name_th</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>name_en</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>province_id</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>deleted_at</t>
         </is>
@@ -5058,7 +5046,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Khoa Khitchakut</t>
+          <t>Khao Khitchakut</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -6798,7 +6786,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Nong Bunnak</t>
+          <t>Nong Bun Mak</t>
         </is>
       </c>
       <c r="D220" t="n">
@@ -7668,7 +7656,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Din Daeng</t>
+          <t>Non Din Daeng</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -10592,12 +10580,12 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>เซกา</t>
+          <t>พรเจริญ</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Seka</t>
+          <t>Phon Charoen</t>
         </is>
       </c>
       <c r="D351" t="n">
@@ -10610,7 +10598,7 @@
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>2025-09-20T06:31:26.000+07:00</t>
+          <t>2026-09-29T00:00:00.000+07:00</t>
         </is>
       </c>
       <c r="G351" t="inlineStr"/>
@@ -10650,12 +10638,12 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>พรเจริญ</t>
+          <t>เซกา</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Phon Charoen</t>
+          <t>Seka</t>
         </is>
       </c>
       <c r="D353" t="n">
@@ -10668,7 +10656,7 @@
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>2025-09-20T06:31:26.000+07:00</t>
+          <t>2026-09-29T00:00:00.000+07:00</t>
         </is>
       </c>
       <c r="G353" t="inlineStr"/>
@@ -10679,12 +10667,12 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>ศรีวิไล</t>
+          <t>ปากคาด</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Si Wilai</t>
+          <t>Pak Khat</t>
         </is>
       </c>
       <c r="D354" t="n">
@@ -10697,7 +10685,7 @@
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>2025-09-20T06:31:26.000+07:00</t>
+          <t>2026-09-29T00:00:00.000+07:00</t>
         </is>
       </c>
       <c r="G354" t="inlineStr"/>
@@ -10737,12 +10725,12 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>ปากคาด</t>
+          <t>ศรีวิไล</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>Pak Khat</t>
+          <t>Si Wilai</t>
         </is>
       </c>
       <c r="D356" t="n">
@@ -10755,7 +10743,7 @@
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>2025-09-20T06:31:26.000+07:00</t>
+          <t>2026-09-29T00:00:00.000+07:00</t>
         </is>
       </c>
       <c r="G356" t="inlineStr"/>
@@ -12279,7 +12267,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>rachak-sinlapakhom</t>
+          <t>Prachaksinlapakhom</t>
         </is>
       </c>
       <c r="D409" t="n">
@@ -13091,7 +13079,7 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>Kantharawichai</t>
+          <t>Chiang Yuen</t>
         </is>
       </c>
       <c r="D437" t="n">

</xml_diff>